<commit_message>
Tighten currency format and add override check + pricing range on Calc
Currency switches to $#,##0;($#,##0);- everywhere. Calc now exposes
Override_Check, Low_End_Range (=Final*0.9), and High_End_Range
(=Final*1.1) for partner-discussion views.
</commit_message>
<xml_diff>
--- a/unit_pricing.xlsx
+++ b/unit_pricing.xlsx
@@ -33,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="_($* #,##0.00_);_($* (#,##0.00);_($* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="$#,##0;($#,##0);-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
@@ -1591,7 +1591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1905,6 +1905,39 @@
       </c>
       <c r="B27" s="25">
         <f>IF(ISNUMBER(in_Override),in_Override,B25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Override_Check</t>
+        </is>
+      </c>
+      <c r="B28" s="23">
+        <f>IF(AND(ISNUMBER(in_Override),OR(LEN(in_OverrideReason)=0,LEN(in_Approver)=0)),"Missing override reason","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>Low_End_Range</t>
+        </is>
+      </c>
+      <c r="B29" s="19">
+        <f>B27*0.9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>High_End_Range</t>
+        </is>
+      </c>
+      <c r="B30" s="19">
+        <f>B27*1.1</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Refine pricing model: fix AI double-count, 0.35 multiplier, T&M, snapshot
- Pull AI automation out of the weighted score (weight → 0) and let it
  act purely as a downward discount; renormalize the other 7 factors
  to sum to 100%.
- Switch factor multiplier from linear (0.25·w̄+0.25) to the
  spec's coefficient form: 1 + Mult_Coef·(w̄ − 3). Mult_Coef is a
  named input (default 0.35) so it is a single knob to calibrate.
- Add residual T&M inputs (TM_Hours, TM_Rate) that flow through to
  the subtotal as hours × rate.
- Add Weight_Sum_Check with conditional formatting that flags when
  CalcFactors weights drift off 100%.
- Extend Calibration with a full audit snapshot (tiers, 8 scores,
  T&M, coefficient, proposed price) and add a log-row block on Calc
  that the user copies → pastes values onto the next Calibration row.
</commit_message>
<xml_diff>
--- a/unit_pricing.xlsx
+++ b/unit_pricing.xlsx
@@ -25,6 +25,9 @@
     <definedName name="in_Override">Inputs!$B$10</definedName>
     <definedName name="in_OverrideReason">Inputs!$B$11</definedName>
     <definedName name="in_Approver">Inputs!$B$12</definedName>
+    <definedName name="in_TMHours">Inputs!$B$13</definedName>
+    <definedName name="in_TMRate">Inputs!$B$14</definedName>
+    <definedName name="in_MultCoef">Inputs!$B$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,12 +35,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0;($#,##0);-"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,6 +82,11 @@
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
     </font>
   </fonts>
   <fills count="6">
@@ -134,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -155,21 +164,26 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -185,6 +199,17 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00F4CCCC"/>
@@ -328,20 +353,33 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Calibration" displayName="Calibration" ref="A1:K2" headerRowCount="1">
-  <autoFilter ref="A1:K2"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Calibration" displayName="Calibration" ref="A1:X2" headerRowCount="1">
+  <autoFilter ref="A1:X2"/>
+  <tableColumns count="24">
     <tableColumn id="1" name="Matter_ID"/>
     <tableColumn id="2" name="Matter_Name"/>
     <tableColumn id="3" name="Deliverable_Type"/>
-    <tableColumn id="4" name="Proposed_Unit_Price"/>
-    <tableColumn id="5" name="Actual_Final_Price"/>
-    <tableColumn id="6" name="Actual_Effort_Cost"/>
-    <tableColumn id="7" name="Margin_%"/>
-    <tableColumn id="8" name="Partner_Feedback"/>
-    <tableColumn id="9" name="Client_Reaction"/>
-    <tableColumn id="10" name="Adjustment_Needed"/>
-    <tableColumn id="11" name="Notes"/>
+    <tableColumn id="4" name="Tech_Tier"/>
+    <tableColumn id="5" name="Token_Tier"/>
+    <tableColumn id="6" name="Score_TechCplx"/>
+    <tableColumn id="7" name="Score_EconRisk"/>
+    <tableColumn id="8" name="Score_Controversy"/>
+    <tableColumn id="9" name="Score_Rigor"/>
+    <tableColumn id="10" name="Score_Scope"/>
+    <tableColumn id="11" name="Score_DataQ"/>
+    <tableColumn id="12" name="Score_DataSens"/>
+    <tableColumn id="13" name="Score_AI"/>
+    <tableColumn id="14" name="TM_Hours"/>
+    <tableColumn id="15" name="TM_Rate"/>
+    <tableColumn id="16" name="Mult_Coef"/>
+    <tableColumn id="17" name="Proposed_Unit_Price"/>
+    <tableColumn id="18" name="Actual_Final_Price"/>
+    <tableColumn id="19" name="Actual_Effort_Cost"/>
+    <tableColumn id="20" name="Margin_%"/>
+    <tableColumn id="21" name="Partner_Feedback"/>
+    <tableColumn id="22" name="Client_Reaction"/>
+    <tableColumn id="23" name="Adjustment_Needed"/>
+    <tableColumn id="24" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -636,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -662,145 +700,176 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>a tech-stack tier, a token-usage tier, and an AI-automation discount.</t>
+          <t>a tech-stack tier, a token-usage tier, residual T&amp;M, and an</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AI-automation discount.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Convention:</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Blue font = input (editable)</t>
+          <t>Convention:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Blue font = input (editable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • Black font = formula (do not overwrite)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Workflow:</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1. Pick deliverable on the Inputs tab.</t>
+          <t>Workflow:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2. Assign scores on the Calc tab (1, 3, or 5 per factor).</t>
+          <t xml:space="preserve">  1. Fill Inputs: matter, deliverable, tiers, T&amp;M hours/rate.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Read the calculated Unit Price on the Calc tab.</t>
+          <t xml:space="preserve">  2. Assign 7 scores on Calc (1, 3, or 5) — AI is a discount only.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. If overridden, populate Override_Reason and Approver on Inputs.</t>
+          <t xml:space="preserve">  3. Read Final Unit Price (highlighted) and Low/High range.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5. Log outcomes on the Calibration tab after the matter closes.</t>
+          <t xml:space="preserve">  4. If overriding, populate Override_Price, Override_Reason, Approver.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5. Copy the Calc snapshot row → paste values onto next Calibration row.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Scoring rule (see Factors tab):</t>
+          <t xml:space="preserve">  6. After the matter closes, fill Actual_Final_Price / Actual_Effort_Cost.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • 3 = baseline</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 1 and 5 require explanation</t>
+          <t>Scoring rule (see Factors tab):</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • AI automation is a downward adjustment only</t>
+          <t xml:space="preserve">  • 3 = baseline</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 1 and 5 require explanation</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Pilot:</t>
+          <t xml:space="preserve">  • AI automation is a downward adjustment only</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Run 10-20 recent matters through the file:</t>
-        </is>
-      </c>
+      <c r="A23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    pick deliverable → assign scores → calculate price →</t>
+          <t>Model knobs (in order to calibrate):</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">    compare to partner's proposal → compare to actual cost → adjust</t>
+          <t xml:space="preserve">  1. Base deliverable prices (Deliverables tab)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Adjust order: base deliverable price → weights → tech/token tiers.</t>
+          <t xml:space="preserve">  2. Tech / Token tiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. Multiplier coefficient (Inputs!Mult_Coef, default 0.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4. Factor weights (Calc!CalcFactors) — must sum to 100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Pilot: run 10-20 recent matters through the file;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>compare to partner's proposal and actual cost; adjust in the order above.</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1568,6 +1637,36 @@
         </is>
       </c>
       <c r="B12" s="13" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>TM_Hours</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>TM_Rate</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Mult_Coef</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>0.35</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -1591,13 +1690,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1613,7 +1724,7 @@
           <t>Matter:</t>
         </is>
       </c>
-      <c r="B3" s="16">
+      <c r="B3" s="18">
         <f>in_MatterName</f>
         <v/>
       </c>
@@ -1624,7 +1735,7 @@
           <t>Deliverable:</t>
         </is>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="18">
         <f>in_Deliverable</f>
         <v/>
       </c>
@@ -1657,13 +1768,13 @@
           <t>Technical complexity / guidance profile</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
-        <v>0.2</v>
+      <c r="B7" s="19" t="n">
+        <v>0.21</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="20">
         <f>[@Weight]*[@Score]</f>
         <v/>
       </c>
@@ -1674,13 +1785,13 @@
           <t>Economic / stakeholder risk</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n">
-        <v>0.15</v>
+      <c r="B8" s="19" t="n">
+        <v>0.16</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="20">
         <f>[@Weight]*[@Score]</f>
         <v/>
       </c>
@@ -1691,13 +1802,13 @@
           <t>Controversy risk</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n">
-        <v>0.15</v>
+      <c r="B9" s="19" t="n">
+        <v>0.16</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="20">
         <f>[@Weight]*[@Score]</f>
         <v/>
       </c>
@@ -1708,13 +1819,13 @@
           <t>Deliverable rigor</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n">
-        <v>0.15</v>
+      <c r="B10" s="19" t="n">
+        <v>0.16</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="20">
         <f>[@Weight]*[@Score]</f>
         <v/>
       </c>
@@ -1725,13 +1836,13 @@
           <t>Scope breadth</t>
         </is>
       </c>
-      <c r="B11" s="17" t="n">
-        <v>0.1</v>
+      <c r="B11" s="19" t="n">
+        <v>0.11</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="20">
         <f>[@Weight]*[@Score]</f>
         <v/>
       </c>
@@ -1742,13 +1853,13 @@
           <t>Data quality / accessibility</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="19" t="n">
         <v>0.1</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="20">
         <f>[@Weight]*[@Score]</f>
         <v/>
       </c>
@@ -1759,13 +1870,13 @@
           <t>Data sensitivity / governance burden</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="19" t="n">
         <v>0.1</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="18">
+      <c r="D13" s="20">
         <f>[@Weight]*[@Score]</f>
         <v/>
       </c>
@@ -1776,13 +1887,13 @@
           <t>AI automation level</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n">
-        <v>0.05</v>
+      <c r="B14" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="18">
+      <c r="D14" s="20">
         <f>[@Weight]*[@Score]</f>
         <v/>
       </c>
@@ -1793,7 +1904,7 @@
           <t>Weighted factor score (w̄)</t>
         </is>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="20">
         <f>SUMPRODUCT(CalcFactors[Weight],CalcFactors[Score])</f>
         <v/>
       </c>
@@ -1801,143 +1912,362 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Factor multiplier (0.5 at w̄=1, 1.0 at 3, 1.5 at 5)</t>
-        </is>
-      </c>
-      <c r="B18" s="18">
-        <f>0.25*B17+0.25</f>
+          <t>Multiplier coefficient</t>
+        </is>
+      </c>
+      <c r="B18" s="20">
+        <f>in_MultCoef</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Base deliverable price</t>
-        </is>
-      </c>
-      <c r="B19" s="19">
-        <f>VLOOKUP(in_Deliverable,Deliverables[[Deliverable_Name]:[Base_Unit_Price]],2,FALSE)</f>
+          <t>Factor multiplier = 1 + coef × (w̄ − 3)</t>
+        </is>
+      </c>
+      <c r="B19" s="20">
+        <f>1+B18*(B17-3)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Tech multiplier</t>
-        </is>
-      </c>
-      <c r="B20" s="20">
-        <f>VLOOKUP(in_TechTier,TechTable[[Tech_Tier]:[Multiplier]],3,FALSE)</f>
+          <t>Base deliverable price</t>
+        </is>
+      </c>
+      <c r="B20" s="21">
+        <f>VLOOKUP(in_Deliverable,Deliverables[[Deliverable_Name]:[Base_Unit_Price]],2,FALSE)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Token add-on</t>
-        </is>
-      </c>
-      <c r="B21" s="19">
-        <f>VLOOKUP(in_TokenTier,TokenTable[[Token_Tier]:[Token_Cost]],3,FALSE)</f>
+          <t>Tech multiplier</t>
+        </is>
+      </c>
+      <c r="B21" s="22">
+        <f>VLOOKUP(in_TechTier,TechTable[[Tech_Tier]:[Multiplier]],3,FALSE)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>AI automation score (1-5)</t>
+          <t>Token add-on</t>
         </is>
       </c>
       <c r="B22" s="21">
-        <f>INDEX(CalcFactors[Score],MATCH("AI automation level",CalcFactors[Factor_Name],0))</f>
+        <f>VLOOKUP(in_TokenTier,TokenTable[[Token_Tier]:[Token_Cost]],3,FALSE)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>AI automation discount (downward only)</t>
-        </is>
-      </c>
-      <c r="B23" s="22">
-        <f>MAX(0,(B22-3)/2)*0.15</f>
+          <t>Residual T&amp;M hours</t>
+        </is>
+      </c>
+      <c r="B23" s="23">
+        <f>in_TMHours</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Subtotal (base × factor × tech + token)</t>
-        </is>
-      </c>
-      <c r="B24" s="19">
-        <f>B19*B18*B20+B21</f>
+          <t>Residual T&amp;M rate</t>
+        </is>
+      </c>
+      <c r="B24" s="21">
+        <f>in_TMRate</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>Unit Price (calculated)</t>
-        </is>
-      </c>
-      <c r="B25" s="19">
-        <f>B24*(1-B23)</f>
+          <t>Residual T&amp;M cost</t>
+        </is>
+      </c>
+      <c r="B25" s="21">
+        <f>B23*B24</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Override in effect?</t>
-        </is>
-      </c>
-      <c r="B26" s="23">
-        <f>IF(ISNUMBER(in_Override),"YES","no")</f>
+          <t>AI automation score (1-5)</t>
+        </is>
+      </c>
+      <c r="B26" s="24">
+        <f>INDEX(CalcFactors[Score],MATCH("AI automation level",CalcFactors[Factor_Name],0))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="24" t="inlineStr">
-        <is>
-          <t>Final Unit Price</t>
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>AI automation discount (downward only)</t>
         </is>
       </c>
       <c r="B27" s="25">
-        <f>IF(ISNUMBER(in_Override),in_Override,B25)</f>
+        <f>MAX(0,(B26-3)/2)*0.15</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>Override_Check</t>
-        </is>
-      </c>
-      <c r="B28" s="23">
-        <f>IF(AND(ISNUMBER(in_Override),OR(LEN(in_OverrideReason)=0,LEN(in_Approver)=0)),"Missing override reason","OK")</f>
+          <t>Subtotal (base × factor × tech + token + T&amp;M)</t>
+        </is>
+      </c>
+      <c r="B28" s="21">
+        <f>B20*B19*B21+B22+B25</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>Low_End_Range</t>
-        </is>
-      </c>
-      <c r="B29" s="19">
-        <f>B27*0.9</f>
+          <t>Unit Price (calculated)</t>
+        </is>
+      </c>
+      <c r="B29" s="21">
+        <f>B28*(1-B27)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
+          <t>Override in effect?</t>
+        </is>
+      </c>
+      <c r="B30" s="26">
+        <f>IF(ISNUMBER(in_Override),"YES","no")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>Final Unit Price</t>
+        </is>
+      </c>
+      <c r="B31" s="28">
+        <f>IF(ISNUMBER(in_Override),in_Override,B29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Override_Check</t>
+        </is>
+      </c>
+      <c r="B32" s="26">
+        <f>IF(AND(ISNUMBER(in_Override),OR(LEN(in_OverrideReason)=0,LEN(in_Approver)=0)),"Missing override reason","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>Low_End_Range</t>
+        </is>
+      </c>
+      <c r="B33" s="21">
+        <f>B31*0.9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
           <t>High_End_Range</t>
         </is>
       </c>
-      <c r="B30" s="19">
-        <f>B27*1.1</f>
+      <c r="B34" s="21">
+        <f>B31*1.1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Weight_Sum_Check (must = 100%)</t>
+        </is>
+      </c>
+      <c r="B35" s="25">
+        <f>SUM(CalcFactors[Weight])</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>Calibration snapshot — copy row below, paste values onto next Calibration row:</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>Matter_ID</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>Matter_Name</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="inlineStr">
+        <is>
+          <t>Deliverable_Type</t>
+        </is>
+      </c>
+      <c r="D38" s="30" t="inlineStr">
+        <is>
+          <t>Tech_Tier</t>
+        </is>
+      </c>
+      <c r="E38" s="30" t="inlineStr">
+        <is>
+          <t>Token_Tier</t>
+        </is>
+      </c>
+      <c r="F38" s="30" t="inlineStr">
+        <is>
+          <t>Score_TechCplx</t>
+        </is>
+      </c>
+      <c r="G38" s="30" t="inlineStr">
+        <is>
+          <t>Score_EconRisk</t>
+        </is>
+      </c>
+      <c r="H38" s="30" t="inlineStr">
+        <is>
+          <t>Score_Controversy</t>
+        </is>
+      </c>
+      <c r="I38" s="30" t="inlineStr">
+        <is>
+          <t>Score_Rigor</t>
+        </is>
+      </c>
+      <c r="J38" s="30" t="inlineStr">
+        <is>
+          <t>Score_Scope</t>
+        </is>
+      </c>
+      <c r="K38" s="30" t="inlineStr">
+        <is>
+          <t>Score_DataQ</t>
+        </is>
+      </c>
+      <c r="L38" s="30" t="inlineStr">
+        <is>
+          <t>Score_DataSens</t>
+        </is>
+      </c>
+      <c r="M38" s="30" t="inlineStr">
+        <is>
+          <t>Score_AI</t>
+        </is>
+      </c>
+      <c r="N38" s="30" t="inlineStr">
+        <is>
+          <t>TM_Hours</t>
+        </is>
+      </c>
+      <c r="O38" s="30" t="inlineStr">
+        <is>
+          <t>TM_Rate</t>
+        </is>
+      </c>
+      <c r="P38" s="30" t="inlineStr">
+        <is>
+          <t>Mult_Coef</t>
+        </is>
+      </c>
+      <c r="Q38" s="30" t="inlineStr">
+        <is>
+          <t>Proposed_Unit_Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="26">
+        <f>in_MatterID</f>
+        <v/>
+      </c>
+      <c r="B39" s="26">
+        <f>in_MatterName</f>
+        <v/>
+      </c>
+      <c r="C39" s="26">
+        <f>in_Deliverable</f>
+        <v/>
+      </c>
+      <c r="D39" s="26">
+        <f>in_TechTier</f>
+        <v/>
+      </c>
+      <c r="E39" s="26">
+        <f>in_TokenTier</f>
+        <v/>
+      </c>
+      <c r="F39" s="24">
+        <f>INDEX(CalcFactors[Score],1)</f>
+        <v/>
+      </c>
+      <c r="G39" s="24">
+        <f>INDEX(CalcFactors[Score],2)</f>
+        <v/>
+      </c>
+      <c r="H39" s="24">
+        <f>INDEX(CalcFactors[Score],3)</f>
+        <v/>
+      </c>
+      <c r="I39" s="24">
+        <f>INDEX(CalcFactors[Score],4)</f>
+        <v/>
+      </c>
+      <c r="J39" s="24">
+        <f>INDEX(CalcFactors[Score],5)</f>
+        <v/>
+      </c>
+      <c r="K39" s="24">
+        <f>INDEX(CalcFactors[Score],6)</f>
+        <v/>
+      </c>
+      <c r="L39" s="24">
+        <f>INDEX(CalcFactors[Score],7)</f>
+        <v/>
+      </c>
+      <c r="M39" s="24">
+        <f>INDEX(CalcFactors[Score],8)</f>
+        <v/>
+      </c>
+      <c r="N39" s="23">
+        <f>in_TMHours</f>
+        <v/>
+      </c>
+      <c r="O39" s="21">
+        <f>in_TMRate</f>
+        <v/>
+      </c>
+      <c r="P39" s="20">
+        <f>in_MultCoef</f>
+        <v/>
+      </c>
+      <c r="Q39" s="21">
+        <f>B31</f>
         <v/>
       </c>
     </row>
@@ -1951,6 +2281,11 @@
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
       <formula>4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B35">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>ROUND(B35,4)&lt;&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1966,20 +2301,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2000,40 +2348,105 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Tech_Tier</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Token_Tier</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Score_TechCplx</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Score_EconRisk</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Score_Controversy</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Score_Rigor</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Score_Scope</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Score_DataQ</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Score_DataSens</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Score_AI</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>TM_Hours</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>TM_Rate</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Mult_Coef</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
           <t>Proposed_Unit_Price</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>Actual_Final_Price</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>Actual_Effort_Cost</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>Margin_%</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>Partner_Feedback</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>Client_Reaction</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>Adjustment_Needed</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2043,17 +2456,30 @@
       <c r="A2" s="3" t="n"/>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="22">
-        <f>IFERROR(([@Actual_Final_Price]-[@Actual_Effort_Cost])/[@Actual_Final_Price],0)</f>
-        <v/>
-      </c>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="4" t="n"/>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="4" t="n"/>
+      <c r="R2" s="4" t="n"/>
+      <c r="S2" s="4" t="n"/>
+      <c r="T2" s="25">
+        <f>IFERROR(([@Actual_Final_Price]-[@Actual_Effort_Cost])/[@Actual_Final_Price],0)</f>
+        <v/>
+      </c>
+      <c r="U2" s="3" t="n"/>
+      <c r="V2" s="3" t="n"/>
+      <c r="W2" s="3" t="n"/>
+      <c r="X2" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>